<commit_message>
docs: move the batch MVP test host to a GCP VM on a private VPC path
- S1-04: the test host is one Compute Engine VM (e2-standard-8, no
  external IP, IAP SSH, Cloud NAT outbound) with the same Compose stack.
- S1-02: the API key stays in all environments. The test host uses a
  private VPC path and a firewall rule; AWS keeps the egress IP allowlist.
- S1-06, S1-11, Sprint 2 ports: VPC firewall rules and IAP instead of
  public IP allowlists and a bastion host.
- S3-06: also test the internet path from a GCP job through Cloud NAT to
  the test AWS cluster, because the test host no longer tests it.
- Private DNS name under a company domain for SSO (S3-07).
</commit_message>
<xml_diff>
--- a/changes/2026-10-02-batch-monitoring-mvp/model_monitoring_issues.xlsx
+++ b/changes/2026-10-02-batch-monitoring-mvp/model_monitoring_issues.xlsx
@@ -1809,19 +1809,21 @@
 additive migration in backend/app/db.py. A stored row never changes. The trace ID comes
 from the traceparent header through the OTel context (S1-05 part B). The backend stores it
 with the row.
-Authentication: a static API key now
-There is no VPN between GCP and AWS yet. Thus the request goes across the internet. Three
-layers protect it:
-Layer | How | Owner
-API key | Authorization: Bearer &lt;key&gt;. A random key of at least 32 bytes for this use case. The GCP job reads it from Secret Manager. The backend stores only its SHA-256 hash and compares in constant time. | Backend + GCP developer
-Encryption | HTTPS only, so that the key is never visible on the network (S1-04) | Platform
-Network | The firewall allows only the egress IP of the GCP job, for example a Cloud NAT static IP (S1-04) | Your team
+Authentication: a static API key in all environments (decided 2026-10-05)
+The test host is in GCP (S1-04). There, the request stays on a private VPC path. In
+Sprint 4, the jobs send to AWS, and the request goes across the internet, because there
+is no VPN between GCP and AWS. The API key is the same in the two environments. Thus the
+test on GCP proves the method that production uses. Three layers protect the request:
+Layer | Test host (GCP, Sprints 1 to 3) | Production (AWS, Sprint 4) | Owner
+API key | Authorization: Bearer &lt;key&gt;. A random key of at least 32 bytes for this use case. The GCP job reads it from Secret Manager. The backend stores only its SHA-256 hash and compares in constant time. | The same | Backend + GCP developer
+Encryption | HTTPS only, with a private CA certificate for the private DNS name (S1-04) | HTTPS only (S4-01) | Platform
+Network | Private VPC path. A VPC firewall rule allows port 443 only from the network ranges of the GCP jobs. The VM has no public IP. (S1-04) | The AWS security rules allow only the egress IPs of the GCP jobs, for example Cloud NAT static IPs (S4-01) | Your team
 Other options:
 Option | Shared secret | Work | Decision
-Static API key + HTTPS + IP allowlist | Yes | Low. The same method as the existing tokens of the monitor. | Selected
+Static API key + HTTPS + network rules | Yes | Low. The same method as the existing tokens of the monitor. | Selected for GCP and for AWS
 Google service-account identity token: the job gets a token that Google signs. The backend examines the signature and the service-account email. | No | Medium. It needs the google-auth package. | Not in October. Only if security requires it (S1-08).
 Mutual TLS | No | High. Each job needs a client certificate. | Not planned
-VPN or private link | — | Depends on the network team | Not available yet</t>
+VPN or private link between GCP and AWS | — | Depends on the network team | Not available yet. The test host does not need it, because it is in GCP.</t>
         </is>
       </c>
       <c r="J3" s="21" t="inlineStr">
@@ -1950,7 +1952,7 @@
       </c>
       <c r="C5" s="21" t="inlineStr">
         <is>
-          <t>Deploy the monitor backend to a test host that GCP can reach</t>
+          <t>Deploy the monitor backend to a test host in GCP</t>
         </is>
       </c>
       <c r="D5" s="21" t="inlineStr">
@@ -1980,39 +1982,59 @@
       </c>
       <c r="I5" s="21" t="inlineStr">
         <is>
-          <t>What: Install the monitor backend, its database and the Collector (S1-06) on a test host
-that the GCP dev project can reach.
-Prerequisites (ask the network team first)
+          <t>What: Make one Compute Engine VM in GCP (decided 2026-10-05). Install the monitor
+backend, its database and the Collector (S1-06) on it with Docker Compose. The GCP jobs
+reach the VM on a private VPC path. The VM has no public IP. In Sprint 2, Langfuse comes on
+the same VM (S2-03).
+Prerequisites (ask the network team and the GCP owner first)
 Question | Why it is important | Owner
-Where does the test host run (AWS account, server or other)? | It decides the firewall and the certificate options | Your team
-How does the network allow traffic between GCP and the host now? | There is no VPN yet. The requests go across the internet. | Network team
-Can port 443 open for one front door (S1-06)? | The API and the Collector both use it. One port, one certificate, one allowlist. | Network team
-What is the egress IP of the GCP job, for example a Cloud NAT static IP? | The firewall allowlist (S1-02) | GCP developer
-Is there a public DNS name for the host? | A public certificate needs it | Your team
-Do we use a public CA certificate, or a private or self-signed certificate? | See the table below | Your team
-Certificate options. Both give real HTTPS.
-Option | Needs | On the GCP job
-Public CA (for example Let's Encrypt or AWS Certificate Manager) | A public DNS name, and a method to prove that you own it | Nothing. The job trusts it by default.
-Private CA or self-signed | Nothing public. We make the certificate and replace it before it expires. | The job trusts our CA file (S1-03). The verification stays on.
-Plain HTTP is not allowed, because the API key would go across the network without encryption.</t>
+Which GCP project and billing account hold the VM? | The owner of the cost and of the access | Your team
+How does the VM network connect to the job projects: the same VPC, Shared VPC, or VPC peering? | The private path from the jobs to the VM | Network team
+Where does each job run: Cloud Run jobs, GKE, Compute Engine, Vertex AI or Dataflow? | Cloud Run and serverless jobs need Direct VPC egress or a Serverless VPC Access connector to reach an internal IP. Record the runtime of each job in S1-09. | GCP developer
+What are the network ranges of the jobs? | The VPC firewall rule for port 443 (S1-02, S1-06) | Network team
+Which private DNS name does the VM get? | A Cloud DNS private zone that the job VPC can see. Use a name under a company domain, because SSO needs it later (S3-07). | Your team
+Can the VM reach the company LiteLLM proxy? | The judge (S1-12, S2-09) | Network team
+How do the staff reach the VPC from the office: the company VPN or Interconnect to GCP? | The dashboard and Langfuse from Sprint 2 (Sprint 2 prerequisites) | Network team
+The VM
+Item | Setting
+Machine | e2-standard-8 (8 vCPU, 32 GiB), the recommended size of the Sprint 2 prerequisites. It is large enough for Langfuse. Thus no resize is necessary in Sprint 2.
+Disk | 200 GiB pd-balanced. A daily snapshot schedule that keeps 7 snapshots.
+Image | Ubuntu 24.04 LTS, Shielded VM on
+Network | No external IP. Cloud NAT for outbound traffic only (Docker images, operating-system updates).
+Service account | A dedicated account with only the roles that the VM needs, for example log and metric writer. Do not use the default Compute Engine service account.
+SSH | Only through IAP: gcloud compute ssh &lt;vm&gt; --tunnel-through-iap. The firewall allows port 22 only from the IAP range 35.235.240.0/20.
+VPC firewall rules (ingress)
+Port | From | For
+443 | The network ranges of the GCP jobs | The API and the Collector (S1-06)
+8443, 3443 | The staff network ranges (from Sprint 2) | The dashboard and Langfuse
+22 | 35.235.240.0/20 (IAP) | SSH for platform and developers (S1-11)
+All other ports | — | Refused. The database ports are never open.
+Certificate. The name is private. Thus a public CA cannot sign it. Make a private CA
+and a certificate for the private DNS name. Replace the certificate before it expires. The
+job trusts the CA file (S1-03). The verification stays on. Google Certificate Authority
+Service is a paid service. Do not use it without a plan entry. Plain HTTP is not allowed.</t>
         </is>
       </c>
       <c r="J5" s="21" t="inlineStr">
         <is>
           <t>• The answers to the prerequisites are in this issue.
-• The monitor backend, PostgreSQL and the Collector run on the test host.
-• The API uses HTTPS (public or private CA). Plain HTTP is refused.
-• Only the GCP egress IP can reach the API and the OTLP endpoint. The database port is closed to the internet.
+• The VM exists with the settings in the table. It has no external IP.
+• The monitor backend, PostgreSQL and the Collector run on the VM.
+• The private DNS name resolves from the job VPC to the internal IP of the VM.
+• The API uses HTTPS with the private CA certificate. Plain HTTP is refused.
+• Only the network ranges of the jobs can reach port 443. The database ports are closed.
+• SSH works only through IAP.
 • The API key and the other secrets are host secrets. They are not in the repository.</t>
         </is>
       </c>
       <c r="K5" s="21" t="inlineStr">
         <is>
-          <t>1. From the GCP dev project: curl https://&lt;test-host&gt;/api/health returns 200. Use --cacert for a private CA.
-2. From an IP that is not on the allowlist: the connection is refused.
+          <t>1. From the GCP dev project, on the job runtime: curl --cacert &lt;ca-file&gt; https://&lt;private-dns-name&gt;/api/health returns 200.
+2. From a network range that is not in the firewall rule: the connection is refused or times out.
 3. POST /api/batch/runs without a key returns 401.
-4. A port scan from the internet shows only the agreed ports.
-5. If the host is late: the GCP developer saves a real body to a file. We send it to the local stack and record that the real delivery was not tested.</t>
+4. gcloud compute instances describe &lt;vm&gt; shows no external IP. The private DNS name does not resolve from the internet.
+5. gcloud compute ssh &lt;vm&gt; --tunnel-through-iap works. SSH to the internal IP from outside the VPC does not work.
+6. If the VM is late: the GCP developer saves a real body to a file. We send it to the local stack and record that the real delivery was not tested.</t>
         </is>
       </c>
       <c r="L5" s="22" t="inlineStr">
@@ -2151,14 +2173,15 @@
 On the test host, put one reverse proxy (the front door) in front of the backend and the
 Collector:
 Path | Goes to | Who calls it | Protection
-https://&lt;host&gt;/api/batch/runs and https://&lt;host&gt;/api/health | Backend | GCP job | API key, IP allowlist
-https://&lt;host&gt;/otlp/* | Collector | GCP job | OTLP token, IP allowlist
+https://&lt;host&gt;/api/batch/runs and https://&lt;host&gt;/api/health | Backend | GCP job | API key, VPC firewall rule
+https://&lt;host&gt;/otlp/* | Collector | GCP job | OTLP token, VPC firewall rule
 Other paths on port 443, for example /api/live/* | Nothing. The front door returns 404. | — | The dashboard data is not available to GCP (S3-07)
-Private network inside the host | Collector | Backend | Not open to the internet
-The firewall opens only port 443. The front door has one certificate (S1-04).
-From Sprint 2, the same front door also serves the staff: the dashboard on port 8443 and
-Langfuse on port 3443, with a separate allowlist for the office or VPN IPs (Sprint 2
-prerequisites). From Sprint 3, the staff also log in with SSO (S3-07).</t>
+Docker network inside the VM | Collector | Backend | Not open outside the VM
+&lt;host&gt; is the private DNS name of the VM (S1-04). The VPC firewall opens port 443 only
+for the network ranges of the GCP jobs. The front door has one certificate (S1-04). From
+Sprint 2, the same front door also serves the staff: the dashboard on port 8443 and Langfuse
+on port 3443, for the staff network ranges only (Sprint 2 prerequisites). From Sprint 3,
+the staff also log in with SSO (S3-07).</t>
         </is>
       </c>
       <c r="J7" s="21" t="inlineStr">
@@ -2166,7 +2189,7 @@
           <t>• docker compose up starts the Collector with a health check.
 • The Collector image has the version from the fixed-versions table. It does not use latest.
 • Spans that come in on OTLP/HTTP appear in the file output.
-• On the test host, the front door is the only public entry. It accepts only port 443 and only the GCP egress IP.
+• On the test host, the front door is the only entry. It has no public IP. Port 443 accepts only the network ranges of the GCP jobs.
 • On port 443, GET /api/live/portfolio returns 404. Only /api/batch/runs, /api/health and /otlp/* reach a service.
 • /otlp/* rejects a request without the correct OTLP token. The OTLP token is different from the API key.
 • The GCP job reads the OTLP token from Secret Manager and sends it with OTEL_EXPORTER_OTLP_HEADERS.
@@ -2179,8 +2202,8 @@
           <t>1. Local: send test spans with telemetrygen traces --otlp-http. Make sure that the file output contains them.
 2. Test host, from the GCP dev project: send test spans to https://&lt;host&gt;/otlp/v1/traces with the token. Make sure that the file output contains them.
 3. Send spans without the token. Make sure that they are rejected.
-4. Send a request from an IP that is not on the allowlist. Make sure that the connection is refused.
-5. From the GCP dev project: curl https://&lt;host&gt;/api/live/portfolio. Make sure that the result is 404.
+4. Send a request from a network range that is not in the firewall rule. Make sure that the connection is refused or times out.
+5. From the GCP dev project: curl --cacert &lt;ca-file&gt; https://&lt;host&gt;/api/live/portfolio. Make sure that the result is 404.
 6. Paired with S1-05: see the test steps in S1-05.</t>
         </is>
       </c>
@@ -2326,10 +2349,10 @@
 The LiteLLM proxy logs: does the proxy store the judge prompts and answers? Where, and for how long? Does it send them to other tools? | S1-12
 The list of PII types that the job replaces with placeholders | S1-03
 The retention period for stored records | S1-02
-An API key on the internet without a VPN, with an IP allowlist | S1-02, S1-04
-The certificate type (public CA or private CA) | S1-04
-The OTLP endpoint that GCP can reach through the front door | S1-06
-Real redacted data on the test host | S1-04
+An API key on a private VPC path in GCP (test host), and later on the internet with an IP allowlist (AWS, Sprint 4) | S1-02, S1-04, S4-01
+The private CA certificate of the test host | S1-04
+The OTLP endpoint that the GCP jobs reach through the front door | S1-06
+Real redacted data on the test host VM in GCP. On the test host, the records stay in GCP. Only the judge calls go to the LiteLLM proxy. | S1-04, S1-12
 Read access to GCP Cloud Logging for the monitor team | S1-01
 Database accounts, and who can read real data | S1-11</t>
         </is>
@@ -2406,7 +2429,8 @@
 Owner | The person who confirms that a run is real
 GCP job and repository | The location of the code that sends the data
 Developer of the job | The person who adds the send step and OTel. This person can be different for each job.
-GCP project and egress IP | The firewall allows only known IP addresses (S1-04). Each project can have a different IP.
+GCP project, job runtime and network range | The private path and the VPC firewall rule to the test host (S1-04). Cloud Run and serverless jobs need VPC egress.
+Egress IP of the job, for example a Cloud NAT static IP | The AWS security rules in Sprint 4 allow only known IP addresses (S4-01). Each project can have a different IP.
 October run dates | The dates when a real run can arrive. If a job does not run in October, book a controlled rerun.
 Batch API or online calls | With the Batch API, latency_s is null
 Approximate number of requests in each run | This number sets the sample size and the load on the LiteLLM proxy (S1-12)
@@ -2419,14 +2443,14 @@
         <is>
           <t>• The table has exactly 10 rows. Each row has a named owner and a named developer.
 • Each use case has at least one October run date, or a booked controlled rerun.
-• Each GCP project has a known egress IP for the allowlist.
+• Each GCP job has a known runtime and network range for the test host, and a known egress IP for AWS.
 • The order of the use cases for Sprints 2 to 4 is agreed.</t>
         </is>
       </c>
       <c r="K10" s="21" t="inlineStr">
         <is>
           <t>1. Each owner confirms their row in the issue comments.
-2. Platform adds all the egress IPs to the allowlist plan (S1-04).
+2. Platform adds the network ranges to the firewall plan of the test host (S1-04), and the egress IPs to the AWS plan (S4-01).
 Risk: The team examined only 6 pipelines in 4 repositories. If the table has fewer
 than 10 real jobs on 9 October, change the October goal and tell the project owner.</t>
         </is>
@@ -2563,7 +2587,7 @@
 Postgres administrator | Person | Platform only | For emergencies only. The backend and the tools do not use it.
 Rules:
 - Keep the passwords as host secrets. Do not put them in the repository or in chat.
-- The database port is not open to the internet. Developers connect through SSH or a bastion host.
+- The database port is not open outside the VM. Developers connect through IAP SSH (gcloud compute ssh &lt;vm&gt; --tunnel-through-iap), then use psql on the VM or an SSH port forward.
 - Remove a developer account when the person leaves the project.
 - Langfuse gets its own database account in S2-03.</t>
         </is>
@@ -2572,7 +2596,7 @@
         <is>
           <t>• Each account in the table exists, with the given permissions.
 • The backend uses monitor_app in DATABASE_URL. It does not use the administrator account.
-• A developer can connect through SSH or the bastion host. A developer cannot connect directly from the internet.
+• A developer can connect through IAP SSH. A developer cannot connect to the database port directly.
 • This issue lists the accounts and their owners. It contains no passwords.</t>
         </is>
       </c>
@@ -2581,7 +2605,7 @@
           <t>1. Start the backend with monitor_app. Make sure that the migrations run and the API stores a run.
 2. Connect as monitor_readonly. Make sure that SELECT works and INSERT fails.
 3. Connect as a dev_&lt;name&gt; account on the test host. Make sure that INSERT fails.
-4. Try to connect to the database port from the internet. Make sure that the connection is refused.</t>
+4. Try to connect to the database port from another VM in the VPC. Make sure that the connection is refused.</t>
         </is>
       </c>
       <c r="L12" s="22" t="inlineStr">
@@ -2639,7 +2663,8 @@
 make sure that the test host can call the proxy. The due date is Friday 9 October, so that
 S2-09 can start on Monday 12 October.
 Question | Why we need it
-The URL of the proxy, for the test host and for AWS | The network path and the firewall rules (S1-04, S4-01)
+The URL of the proxy, for the test host (a VM in a GCP VPC) and for AWS | The network path and the firewall rules (S1-04, S4-01)
+How does the GCP VPC reach the proxy: Interconnect, VPN, or a public endpoint through Cloud NAT? | The test host has no public IP. Its outbound traffic goes through Cloud NAT or a private link.
 The model alias for the judge, and the model behind it: name, version, context length | The judge identity on each score. RAI accepts this model (S2-10).
 Does the model support response_format with type: json_schema? | S2-09 asks for the four scores as JSON with a fixed schema
 Does the model understand Thai well? | Many use cases are in Thai (S1-09)
@@ -2900,8 +2925,8 @@
 GCP spans to the Langfuse OTLP endpoint (/api/public/otel) with the Langfuse project keys.
 Prerequisites (answer after S1-04 is complete)
 Question | Owner
-Is the test host large enough for Langfuse (CPU, memory, disk)? Examine the Langfuse self-hosting requirements. | Platform
-How do the engineers open the Langfuse UI? The front door allows only the GCP IP now. Options: add the office or VPN IP, or use an SSH tunnel. | Network team
+Is the test host VM large enough for Langfuse (CPU, memory, disk)? S1-04 uses e2-standard-8 and 200 GiB. Examine the Langfuse self-hosting requirements. | Platform
+Do the engineers reach port 3443 through the company network path to the VPC? If not, use an IAP tunnel: gcloud compute start-iap-tunnel &lt;vm&gt; 3443. | Network team
 Rules
 - Langfuse uses its own PostgreSQL container and account. It does not share the monitor database (S1-11).
 - Turn off public sign-up in Langfuse. Make one account for each engineer. Langfuse is for engineers. The RAI team uses the dashboard.
@@ -3193,7 +3218,7 @@
 For each job, do these steps:
 1. Add the use case to the YAML registry (S2-01) in a pull request. Set mode: identity_only.
 2. Platform makes the API key with scripts/batch_keys.py and puts it into the GCP Secret Manager of that project.
-3. Platform adds the egress IP of the GCP project to the allowlist.
+3. Platform gives the job a private path to the test host: VPC access for the job runtime, and its network range in the firewall rule (S1-04). Record the egress IP of the job for AWS (S4-01).
 4. The job developer maps the job to the record fields of the standard, as in S1-01.
 5. The job developer adds the send step and the helper file. The job uses the shared OTLP token. It needs no Langfuse key.
 6. Run the job. If the job does not run between 12 and 16 October, use a controlled rerun.
@@ -3821,7 +3846,7 @@
       <c r="I26" s="21" t="inlineStr">
         <is>
           <t>What: Make the Collector safe and reliable before AWS. S1-06 already added the token,
-HTTPS through the front door and the IP allowlist. This issue does not repeat them.
+HTTPS through the front door and the network rules. This issue does not repeat them.
 Addition | Why
 Attribute filter in the Collector | The helper file removes attributes in the GCP job (S2-04). The Collector filter is a second protection, for example for a job that uses an old helper file. Use the same allowlist.
 Memory limit | A large burst of spans cannot stop the Collector
@@ -3986,6 +4011,7 @@
 - The Langfuse accounts. They are for engineers only.
 - One key rotation (S2-01).
 - A request without a key or a token is refused, on the API and on the Collector.
+- The test host VM has no external IP. The VPC firewall rules allow only the ranges in S1-04. The VM uses its own service account, not the default one.
 - The retention periods in the monitor database and in Langfuse (S1-08).</t>
         </is>
       </c>
@@ -4064,7 +4090,11 @@
 Langfuse SSO (S3-07) | SSO settings in the Helm values file. The client secret comes from the Kubernetes secret store. | The same
 Send the RDS and S3 request in Sprint 1 (long-lead requests). If the request is not
 approved by Wednesday 21 October, use plan B. Write the deployment files so that a
-values file selects plan A or plan B.</t>
+values file selects plan A or plan B.
+The first test of the internet path. The test host is in GCP, on a private path
+(S1-04). Thus Sprints 1 and 2 do not test the path that production uses: from a GCP job,
+through its Cloud NAT egress IP, across the internet, to AWS. Test this path here, on the
+test AWS cluster, before Sprint 4.</t>
         </is>
       </c>
       <c r="J29" s="21" t="inlineStr">
@@ -4075,13 +4105,14 @@
 • Secrets come from the Kubernetes secret store. No secret is in the files. This includes LLM_JUDGE_API_KEY, the OAuth client secrets and the OAuth2 Proxy cookie secret.
 • Each service has health checks, resource limits and a rollback step.
 • Backup, restore and rollback steps are written. For plan A, they use the RDS backups.
-• The stack runs on the test AWS Kubernetes cluster, and the smoke test passes.</t>
+• The stack runs on the test AWS Kubernetes cluster, and the smoke test passes.
+• A job runtime in the GCP dev project sends one example run and spans to the test AWS cluster, through its Cloud NAT egress IP. The AWS security rules allow that IP only. A request from another IP is refused.</t>
         </is>
       </c>
       <c r="K29" s="21" t="inlineStr">
         <is>
           <t>1. Validate all the files.
-2. Install the stack on the test AWS Kubernetes cluster. Send one example run and spans from a GCP dev machine. Run scripts/check_trace.py, and make sure that all the items are "found".
+2. Install the stack on the test AWS Kubernetes cluster. Send one example run and spans from the job runtime in the GCP dev project, through Cloud NAT. Run scripts/check_trace.py, and make sure that all the items are "found".
 3. If the test cluster is not available by 19 October, install the stack on a disposable local cluster (for example kind) with plan B, and record that the AWS test was not done.</t>
         </is>
       </c>
@@ -4137,7 +4168,10 @@
         <is>
           <t>What: The staff log in with their company Google Workspace account. Later, the company
 changes to Microsoft Entra ID. Thus the identity provider is a setting only, and a runbook
-describes the change. The IP allowlists stay as a second protection.
+describes the change. The VPC firewall rules for the staff network ranges stay as a second
+protection. The test host uses its private DNS name (S1-04). Google accepts a private name
+under a company domain, because the browser follows the redirect inside the company
+network.
 Part | How | Code change
 Dashboard (port 8443) | OAuth2 Proxy (fixed versions table) in front of the dashboard and its API. Provider google. Only the emails in the allowlist file can enter. | None. The frontend files do not change. The backend port stays private.
 Langfuse (port 3443) | The built-in SSO of Langfuse, with Google. Password login is off. | None. Settings only.
@@ -4178,7 +4212,7 @@
 1. Register the redirect URIs in the two Google OAuth clients: https://&lt;test-host-dns&gt;:8443/oauth2/callback and https://&lt;test-host-dns&gt;:3443/api/auth/callback/google.
 2. Turn on Google login in Langfuse, with password login still on. Make sure that the engineer with the owner role logs in with Google and keeps the owner role (account linking by email, S2-03).
 3. Then set AUTH_DISABLE_USERNAME_PASSWORD=true.
-4. Put OAuth2 Proxy in front of the dashboard. Keep the IP allowlist.
+4. Put OAuth2 Proxy in front of the dashboard. Keep the firewall rules for the staff network ranges.
 Local stack and CI. Use the mock OIDC server (fixed versions table) as the identity
 provider: OAuth2 Proxy with OAUTH2_PROXY_PROVIDER=oidc and
 OAUTH2_PROXY_OIDC_ISSUER_URL=http://mock-oidc:8080/default, and Langfuse with the
@@ -4275,7 +4309,7 @@
 1. Select plan A (RDS and S3) or plan B (in the cluster), from the S3-06 decision.
 2. Replace the test-host front door with the AWS load balancer and ingress. Keep the same paths: /api/batch/runs, /api/health and /otlp/* for GCP, and the dashboard and Langfuse behind SSO for the staff (S3-07).
 3. Use the DNS name and the certificate from the long-lead requests. If they are not available, use the IP address and a private CA certificate. Without a DNS name, Google SSO does not work. Then the dashboard has only the IP allowlist, and the release result records this exception.
-4. Allow the egress IPs of all 10 GCP projects (S1-09) in the AWS security rules.
+4. Allow the egress IPs of all 10 GCP jobs (S1-09) in the AWS security rules. The S3-06 test already proved this path for one job.
 5. Allow a network path from the cluster to the company LiteLLM proxy. Use the AWS virtual key from S1-12.
 6. Add the AWS redirect URIs to the two Google OAuth clients (S3-07).
 7. Do not configure the prototype use cases.
@@ -4354,6 +4388,10 @@
 2. The OTLP endpoint.
 3. The API key. Make a new production key with scripts/batch_keys.py, and put it into the GCP Secret Manager of that project.
 If AWS uses a private CA, the job trusts the new CA file.
+The network path also changes. On the test host, the job used a private VPC path. To AWS,
+the job sends across the internet through its Cloud NAT egress IP. Make sure that the job
+runtime has outbound internet access through Cloud NAT, and that the egress IP is in the AWS
+security rules (S4-01).
 Fallback: Keep the test host running for one week after the change. If AWS has a
 problem, a job can go back to the test host with its old settings.</t>
         </is>
@@ -5287,7 +5325,7 @@
       </c>
       <c r="D2" s="21" t="inlineStr">
         <is>
-          <t>Use the IP address and a private CA certificate, as on the test host</t>
+          <t>Use the IP address and a private CA certificate</t>
         </is>
       </c>
     </row>
@@ -5382,7 +5420,7 @@
     <row r="7">
       <c r="A7" s="21" t="inlineStr">
         <is>
-          <t>DNS name for the test host. Google does not accept an IP address in an SSO redirect URI.</t>
+          <t>A private DNS name for the test host under a company domain, in a Cloud DNS private zone (for example monitor-test.&lt;company domain&gt;). Google does not accept an IP address or a .internal name in an SSO redirect URI. The name does not have to be public.</t>
         </is>
       </c>
       <c r="B7" s="21" t="inlineStr">
@@ -5397,7 +5435,7 @@
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>No SSO on the test host. The dashboard and Langfuse keep only the IP allowlist and the Langfuse accounts. S3-05 records the exception.</t>
+          <t>No SSO on the test host. The dashboard and Langfuse keep only the firewall rules and the Langfuse accounts. S3-05 records the exception.</t>
         </is>
       </c>
     </row>

</xml_diff>